<commit_message>
Notes and timings of 2026 class
</commit_message>
<xml_diff>
--- a/2026_timing.xlsx
+++ b/2026_timing.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pietro.berkes/ogit/aspp/scientific_programming_patterns/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14AFB8F5-4FA0-4048-A885-65D903B282A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7A5598-286D-0C4D-A014-866209EE5DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3260" yWindow="2260" windowWidth="28040" windowHeight="17180" xr2:uid="{EE13F057-85BC-314B-B061-0A02A8805DDF}"/>
+    <workbookView xWindow="1300" yWindow="660" windowWidth="33260" windowHeight="21680" xr2:uid="{EE13F057-85BC-314B-B061-0A02A8805DDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
   <si>
     <t>Expected time</t>
   </si>
   <si>
-    <t>Actual time</t>
-  </si>
-  <si>
     <t>What</t>
   </si>
   <si>
@@ -105,6 +102,30 @@
   </si>
   <si>
     <t xml:space="preserve">Constructor smell </t>
+  </si>
+  <si>
+    <t>Actual time (Start)</t>
+  </si>
+  <si>
+    <t>It was nice to explain the three possible choices for position+dt as part of the Particle class</t>
+  </si>
+  <si>
+    <t>Idea: Phrase exercise as: Go through parameters and functions, and discuss if they belong</t>
+  </si>
+  <si>
+    <t>Very quick because some of it was mentioned in the solution</t>
+  </si>
+  <si>
+    <t>Content of git issue is more informative than text on slide!</t>
+  </si>
+  <si>
+    <t>A few good questions about projects: scratch code for prototyping, log for making sense of project</t>
+  </si>
+  <si>
+    <t>Wrapping up at least 5 min too early</t>
+  </si>
+  <si>
+    <t>Did an improv bit instead</t>
   </si>
 </sst>
 </file>
@@ -478,7 +499,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11432D03-3CA3-CD43-B1BF-03B6D1AC6980}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" customWidth="1"/>
@@ -490,24 +511,24 @@
     <col min="10" max="10" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>0.41666666666666669</v>
       </c>
@@ -516,13 +537,13 @@
         <v>9.9999999999999645</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>0.4236111111111111</v>
       </c>
@@ -531,13 +552,13 @@
         <v>10.000000000000044</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>0.43055555555555558</v>
       </c>
@@ -546,13 +567,13 @@
         <v>14.999999999999947</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>0.44097222222222221</v>
       </c>
@@ -561,13 +582,16 @@
         <v>4.9999999999999822</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>0.44444444444444442</v>
       </c>
@@ -576,13 +600,16 @@
         <v>10.000000000000044</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.45624999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>0.4513888888888889</v>
       </c>
@@ -591,13 +618,16 @@
         <v>15.000000000000027</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.46319444444444446</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>0.46180555555555558</v>
       </c>
@@ -606,13 +636,19 @@
         <v>9.9999999999999645</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.47569444444444442</v>
+      </c>
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>0.46875</v>
       </c>
@@ -621,13 +657,19 @@
         <v>15.000000000000027</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>0.47916666666666669</v>
       </c>
@@ -637,10 +679,13 @@
       </c>
       <c r="C10" s="1"/>
       <c r="D10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.48472222222222222</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>0.5</v>
       </c>
@@ -649,13 +694,13 @@
         <v>9.9999999999999645</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>0.50694444444444442</v>
       </c>
@@ -664,13 +709,16 @@
         <v>15.000000000000107</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+      <c r="H12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>0.51736111111111116</v>
       </c>
@@ -679,13 +727,13 @@
         <v>4.9999999999999822</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>0.52083333333333337</v>
       </c>
@@ -694,13 +742,16 @@
         <v>9.9999999999999645</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>0.52777777777777779</v>
       </c>
@@ -709,13 +760,13 @@
         <v>14.999999999999947</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>0.53819444444444442</v>
       </c>
@@ -724,13 +775,13 @@
         <v>4.9999999999999822</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>0.54166666666666663</v>
       </c>
@@ -739,13 +790,19 @@
         <v>20.000000000000089</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.53749999999999998</v>
+      </c>
+      <c r="H17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>0.55555555555555558</v>
       </c>
@@ -754,13 +811,19 @@
         <v>9.9999999999999645</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.55208333333333337</v>
+      </c>
+      <c r="H18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>0.5625</v>
       </c>
@@ -769,28 +832,28 @@
         <v>0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>0.5625</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B21" s="2"/>
       <c r="C21" s="1"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
     </row>

</xml_diff>

<commit_message>
Add Lisa's LatAm timing
</commit_message>
<xml_diff>
--- a/2026_timing.xlsx
+++ b/2026_timing.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pietro.berkes/ogit/aspp/scientific_programming_patterns/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7A5598-286D-0C4D-A014-866209EE5DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D9AF54-9031-AC4F-87E2-3402BCA53BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1300" yWindow="660" windowWidth="33260" windowHeight="21680" xr2:uid="{EE13F057-85BC-314B-B061-0A02A8805DDF}"/>
   </bookViews>
@@ -542,6 +542,9 @@
       <c r="D2" t="s">
         <v>2</v>
       </c>
+      <c r="E2" s="1">
+        <v>0.42083333333333334</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -557,6 +560,9 @@
       <c r="D3" t="s">
         <v>3</v>
       </c>
+      <c r="E3" s="1">
+        <v>0.42638888888888887</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -572,6 +578,9 @@
       <c r="D4" t="s">
         <v>4</v>
       </c>
+      <c r="E4" s="1">
+        <v>0.43819444444444444</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -699,6 +708,9 @@
       <c r="D11" t="s">
         <v>20</v>
       </c>
+      <c r="E11" s="1">
+        <v>0.50347222222222221</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
@@ -714,6 +726,9 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
+      <c r="E12" s="1">
+        <v>0.51111111111111107</v>
+      </c>
       <c r="H12" t="s">
         <v>25</v>
       </c>
@@ -732,6 +747,9 @@
       <c r="D13" t="s">
         <v>5</v>
       </c>
+      <c r="E13" s="1">
+        <v>0.52430555555555558</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
@@ -746,6 +764,9 @@
       </c>
       <c r="D14" t="s">
         <v>10</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.53125</v>
       </c>
       <c r="H14" t="s">
         <v>28</v>

</xml_diff>